<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-05 Le seau de la sauge
Réécriture vocale example4 : éclat de sauge, énergie vécue, N1.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-05.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, terre mouillée</t>
+          <t>jardin : sauge, goutte froide, terre, caisse, seau rouge, bac d'eau, linge</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut arroser la sauge avec le seau rouge. Aniss a de l'énergie. L'eau touche les chaussures. Ils jouent, ils attendent, Mila demande à papa. La sauge boit.</t>
+          <t>Une goutte froide tient sur la sauge. Sur la feuille, un éclat de sauge brille. Mila veut le seau rouge, maintenant. Aniss saute trop. L'eau part partout. Sourire parti. Elle refuse de foncer. Merci vécu. Ils se passent le seau. Il veut verser tout. Elle s'arrête. Un éclat de sauge tient sur la feuille.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un ver de terre rose traverse le chemin. Il brille. La terre est molle. Elle est sombre. Une caisse sent le bois mouillé. Un seau rouge attend. Papa a de la terre sur une chaussure. Tu vois le ver, Mila ? Oui. Il brille. Maman tord un linge. Le bac est plein d'eau. En ce moment, Mila touche une feuille. La feuille de sauge est un peu rêche. Elle sent fort, un peu comme le savon. Je veux le seau. Pour la sauge. Il est près du bac. Mila marche vers le bac. L'eau tremble. Elle est claire. Aniss arrive en sautant. Il a beaucoup d'énergie. Il tourne. Il s'arrête. Il recommence. Il saute, maman. C'est son énergie. Ce n'est pas une faute. Aniss prend le seau. L'eau bouge. Un peu d'eau touche les chaussures. Le seau. À tour de rôle. Oui. On attend. Aniss tient encore le seau. Il saute un peu. Mila regarde papa.</t>
+          <t>Une goutte froide tient sur la sauge. Elle tremble, ronde et claire. Elle est froide, papa. Tu la vois, Mila ? Oui, papa. La feuille de sauge sent le savon. Ça sent fort, maman. Tu le sens, le savon ? Oui, maman. La terre est molle, un peu sombre. Tes chaussures sont mouillées, Mila ? Un peu, papa. Papa a de la terre sur une chaussure. Tu as vu la terre, Mila ? Oui, papa. Une caisse sent le bois mouillé. Un seau rouge attend près du bac. Le seau est rouge. Il est près du bac ? Oui, maman. Maman tord un linge. Le linge goutte sur la terre. Le bac est plein, Mila ? L'eau tremble. En ce moment, Mila touche la feuille. Sur la feuille, un éclat de sauge brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Je veux le seau, maintenant ! Pour la sauge ? Oui, tout de suite. Avec le seau rouge ? Oui, papa. Mila marche vers le bac. L'eau du bac est claire. Aniss arrive dans le jardin. Il saute trop, trop vite. Le seau ! Aniss ! J'arrive ! Mila prend le seau trop vite. Aniss saute contre le seau. L'eau part partout. Elle mouille les chaussures. Oh. L'eau ! Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Mila ? Oui, papa. Tes mains sont froides, Mila ? Un peu, maman. L'éclat de sauge tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un ver de terre rose traverse le chemin. Il brille. La terre est molle. Elle est sombre. Une caisse sent le bois mouillé. Un seau rouge attend. Papa a de la terre sur une chaussure. Tu vois le ver, Mila ? Oui. Il brille. Maman tord un linge. Le bac est plein d'eau. En ce moment, Mila touche une feuille. La feuille de sauge est un peu rêche. Elle sent fort, un peu comme le savon. Je veux le seau. Pour la sauge. Il est près du bac. Mila marche vers le bac. L'eau tremble. Elle est claire. Aniss arrive en sautant. Il a beaucoup d'énergie. Il tourne. Il s'arrête. Il recommence. Il saute, maman. C'est son énergie. Ce n'est pas une faute. Aniss prend le seau. L'eau bouge. Un peu d'eau touche les chaussures. Le seau. À tour de rôle. Oui. On attend. Aniss tient encore le seau. Il saute un peu. Mila regarde papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte froide tient sur la sauge. Elle tremble, ronde et claire. Elle est froide, papa. Tu la vois, Mila ? Oui, papa. La feuille de sauge sent le savon. Ça sent fort, maman. Tu le sens, le savon ? Oui, maman. La terre est molle, un peu sombre. Tes chaussures sont mouillées, Mila ? Un peu, papa. Papa a de la terre sur une chaussure. Tu as vu la terre, Mila ? Oui, papa. Une caisse sent le bois mouillé. Un seau rouge attend près du bac. Le seau est rouge. Il est près du bac ? Oui, maman. Maman tord un linge. Le linge goutte sur la terre. Le bac est plein, Mila ? L'eau tremble. En ce moment, Mila touche la feuille. Sur la feuille, un &lt;emphasis level="moderate"&gt;éclat de sauge&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Je veux le seau, maintenant ! Pour la sauge ? Oui, tout de suite. Avec le seau rouge ? Oui, papa. Mila marche vers le bac. L'eau du bac est claire. Aniss arrive dans le jardin. Il saute trop, trop vite. Le seau ! Aniss ! J'arrive ! Mila prend le seau trop vite. Aniss saute contre le seau. L'eau part partout. Elle mouille les chaussures. Oh. L'eau ! Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Mila ? Oui, papa. Tes mains sont froides, Mila ? Un peu, maman. L'éclat de sauge tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tania joue au jardin. Maman est près du bac. Ulysse arrive en sautant. Il a beaucoup d'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Il tourne. Il s'arrête. Il recommence. Tania le regarde. Maman dit : beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. Tania hoche la tête. Elle dit : à tour de rôle. Ulysse attend. Puis Tania joue. Puis Ulysse joue. L'énergie est encore là. Ce n'est pas une faute. Ils jouent ensemble.&lt;/slow&gt; [pause]</t>
+          <t>Une goutte froide tient sur la sauge. Elle tremble, ronde et claire. Elle est froide, papa. Tu la vois, Mila ? Oui, papa. La feuille de sauge sent le savon. Ça sent fort, maman. Tu le sens, le savon ? Oui, maman. La terre est molle, un peu sombre. Tes chaussures sont mouillées, Mila ? Un peu, papa. Papa a de la terre sur une chaussure. Tu as vu la terre, Mila ? Oui, papa. Une caisse sent le bois mouillé. Un seau rouge attend près du bac. Le seau est rouge. Il est près du bac ? Oui, maman. Maman tord un linge. Le linge goutte sur la terre. Le bac est plein, Mila ? L'eau tremble. En ce moment, Mila touche la feuille. Sur la feuille, un &lt;emphasis&gt;éclat de sauge&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Je veux le seau, maintenant ! Pour la sauge ? Oui, tout de suite. Avec le seau rouge ? Oui, papa. Mila marche vers le bac. L'eau du bac est claire. Aniss arrive dans le jardin. Il saute trop, trop vite. Le seau ! Aniss ! J'arrive ! Mila prend le seau trop vite. Aniss saute contre le seau. L'eau part partout. Elle mouille les chaussures. Oh. L'eau ! Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Mila ? Oui, papa. Tes mains sont froides, Mila ? Un peu, maman. L'éclat de sauge tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de sauge</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,50 +1319,72 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_seau_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un ver de terre rose traverse le chemin.
-narrateur|Il brille.
-narrateur|La terre est molle.
-narrateur|Elle est sombre.
+          <t>narrateur|Une goutte froide tient sur la sauge.
+narrateur|Elle tremble, ronde et claire.
+enfant-f|Elle est froide, papa.
+papa|Tu la vois, Mila ?
+enfant-f|Oui, papa.
+narrateur|La feuille de sauge sent le savon.
+enfant-f|Ça sent fort, maman.
+maman|Tu le sens, le savon ?
+enfant-f|Oui, maman.
+narrateur|La terre est molle, un peu sombre.
+papa|Tes chaussures sont mouillées, Mila ?
+enfant-f|Un peu, papa.
+narrateur|Papa a de la terre sur une chaussure.
+papa|Tu as vu la terre, Mila ?
+enfant-f|Oui, papa.
 narrateur|Une caisse sent le bois mouillé.
-narrateur|Un seau rouge attend.
-narrateur|Papa a de la terre sur une chaussure.
-papa|Tu vois le ver, Mila ?
-enfant-f|Oui.
-enfant-f|Il brille.
+narrateur|Un seau rouge attend près du bac.
+enfant-f|Le seau est rouge.
+maman|Il est près du bac ?
+enfant-f|Oui, maman.
 narrateur|Maman tord un linge.
-maman|Le bac est plein d'eau.
-narrateur|En ce moment, Mila touche une feuille.
-narrateur|La feuille de sauge est un peu rêche.
-narrateur|Elle sent fort, un peu comme le savon.
-enfant-f|Je veux le seau.
-enfant-f|Pour la sauge.
-maman|Il est près du bac.
+narrateur|Le linge goutte sur la terre.
+papa|Le bac est plein, Mila ?
+enfant-f|L'eau tremble.
+narrateur|En ce moment, Mila touche la feuille.
+narrateur|Sur la feuille, un éclat de sauge brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+enfant-f|Je veux le seau, maintenant !
+maman|Pour la sauge ?
+enfant-f|Oui, tout de suite.
+papa|Avec le seau rouge ?
+enfant-f|Oui, papa.
 narrateur|Mila marche vers le bac.
-narrateur|L'eau tremble.
-narrateur|Elle est claire.
-narrateur|Aniss arrive en sautant.
-narrateur|Il a beaucoup d'énergie.
-narrateur|Il tourne.
-narrateur|Il s'arrête.
-narrateur|Il recommence.
-enfant-f|Il saute, maman.
-maman|C'est son énergie.
-maman|Ce n'est pas une faute.
-narrateur|Aniss prend le seau.
-narrateur|L'eau bouge.
-narrateur|Un peu d'eau touche les chaussures.
-enfant-f|Le seau.
-enfant-f|À tour de rôle.
-papa|Oui.
-papa|On attend.
-narrateur|Aniss tient encore le seau.
-narrateur|Il saute un peu.
-narrateur|Mila regarde papa.</t>
+narrateur|L'eau du bac est claire.
+narrateur|Aniss arrive dans le jardin.
+narrateur|Il saute trop, trop vite.
+copain|Le seau !
+enfant-f|Aniss !
+copain|J'arrive !
+narrateur|Mila prend le seau trop vite.
+narrateur|Aniss saute contre le seau.
+narrateur|L'eau part partout.
+narrateur|Elle mouille les chaussures.
+enfant-f|Oh.
+copain|L'eau !
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Mila ?
+enfant-f|Oui, papa.
+maman|Tes mains sont froides, Mila ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de sauge tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1399,12 +1421,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss a de l'énergie. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ulysse a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1467,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1478,7 +1500,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,11 +1515,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1508,23 +1530,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,7 +1561,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1549,7 +1571,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=aniss_saute_trop_que_peut_on_faire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1582,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila va vers papa. Papa, le seau ? On verse pour la sauge. On attend son tour. Tu peux me demander. On se passe le seau. Aniss tend les mains. Il a encore de l'énergie. Ce n'est pas une faute. On peut attendre. Aniss souffle. Il attend. Mila verse tout doucement. La sauge boit. Ploc. Aniss verse après. Ils jouent. Ils se passent le seau. Une autre goutte tombe. La terre sent fort. Tu veux encore verser, Mila ? Oui. Mila verse. Aniss attend. Chacun son tour. Un oiseau chante tout près. Tu l'as entendu ? Oui, papa. Le ver de terre n'est plus là. La terre a un petit trou brillant. Il est rentré. Il a de l'eau, maintenant.</t>
+          <t>Mila veut le seau, tout de suite. Je verse, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Attends. Aniss recule d'un pas. Oh. Le sourire ne revient pas. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le seau, un instant. Elle écoute le linge qui goutte. Tu veux le seau avec Aniss ? Papa reste à la même hauteur. Tu tiens l'anse ? Aniss ne dit rien, d'abord. Il pose les mains sur le seau. Je le tiens. D'accord. Merci, Mila. Papa a vu les deux, près du bac. La sauge est rêche, sous les doigts. Elle sent le savon. Ils se passent le seau. Aniss tient l'anse, plus près. Mila verse un peu, cette fois. Ploc. Ploc. Tu vois, la sauge ? Oui, papa. Elle boit, Aniss ? Un peu. Mila verse, sans se presser. Aniss suit le seau des yeux. La terre devient plus sombre. Un. Deux. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près de la sauge ? Oui. Tes mains sont mouillées, Mila ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila va vers papa. Papa, le seau ? On verse pour la sauge. On attend son tour. Tu peux me demander. On se passe le seau. Aniss tend les mains. Il a encore de l'énergie. Ce n'est pas une faute. On peut attendre. Aniss souffle. Il attend. Mila verse tout doucement. La sauge boit. Ploc. Aniss verse après. Ils jouent. Ils se passent le seau. Une autre goutte tombe. La terre sent fort. Tu veux encore verser, Mila ? Oui. Mila verse. Aniss attend. Chacun son tour. Un oiseau chante tout près. Tu l'as entendu ? Oui, papa. Le ver de terre n'est plus là. La terre a un petit trou brillant. Il est rentré. Il a de l'eau, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, tout de suite. Je verse, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Attends. Aniss recule d'un pas. Oh. Le sourire ne revient pas. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le seau, un instant. Elle écoute le linge qui goutte. Tu veux le seau avec Aniss ? Papa reste à la même hauteur. Tu tiens l'anse ? Aniss ne dit rien, d'abord. Il pose les mains sur le seau. Je le tiens. D'accord. Merci, Mila. Papa a vu les deux, près du bac. La sauge est rêche, sous les doigts. Elle sent le savon. Ils se passent le seau. Aniss tient l'anse, plus près. Mila verse un peu, cette fois. Ploc. Ploc. Tu vois, la sauge ? Oui, papa. Elle boit, Aniss ? Un peu. Mila verse, sans se presser. Aniss suit le seau des yeux. La terre devient plus sombre. Un. Deux. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près de la sauge ? Oui. Tes mains sont mouillées, Mila ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ulysse a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Tania a joué. Elle a su attendre.&lt;/slow&gt; [pause]</t>
+          <t>Mila veut le &lt;emphasis&gt;seau&lt;/emphasis&gt;, tout de suite. Je verse, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Attends. Aniss recule d'un pas. Oh. Le sourire ne revient pas. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le seau, un instant. Elle écoute le linge qui goutte. Tu veux le seau avec Aniss ? Papa reste à la même hauteur. Tu tiens l'anse ? Aniss ne dit rien, d'abord. Il pose les mains sur le seau. Je le tiens. D'accord. Merci, Mila. Papa a vu les deux, près du bac. La sauge est rêche, sous les doigts. Elle sent le savon. Ils se passent le seau. Aniss tient l'anse, plus près. Mila verse un peu, cette fois. Ploc. Ploc. Tu vois, la sauge ? Oui, papa. Elle boit, Aniss ? Un peu. Mila verse, sans se presser. Aniss suit le seau des yeux. La terre devient plus sombre. Un. Deux. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près de la sauge ? Oui. Tes mains sont mouillées, Mila ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,18 +1661,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1717,47 +1739,59 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_ils_se_passent_le_seau; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila va vers papa.
-enfant-f|Papa, le seau ?
-papa|On verse pour la sauge.
-papa|On attend son tour.
-papa|Tu peux me demander.
-papa|On se passe le seau.
-narrateur|Aniss tend les mains.
-narrateur|Il a encore de l'énergie.
-maman|Ce n'est pas une faute.
-enfant-f|On peut attendre.
-narrateur|Aniss souffle.
-narrateur|Il attend.
-narrateur|Mila verse tout doucement.
-narrateur|La sauge boit.
-narrateur|Ploc.
-narrateur|Aniss verse après.
-narrateur|Ils jouent.
+          <t>narrateur|Mila veut le seau, tout de suite.
+enfant-f|Je verse, maintenant !
+narrateur|Elle avance trop vite vers Aniss.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Attends.
+narrateur|Aniss recule d'un pas.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le seau, un instant.
+narrateur|Elle écoute le linge qui goutte.
+papa|Tu veux le seau avec Aniss ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Tu tiens l'anse ?
+narrateur|Aniss ne dit rien, d'abord.
+narrateur|Il pose les mains sur le seau.
+copain|Je le tiens.
+enfant-f|D'accord.
+papa|Merci, Mila.
+narrateur|Papa a vu les deux, près du bac.
+maman|La sauge est rêche, sous les doigts.
+enfant-f|Elle sent le savon.
 narrateur|Ils se passent le seau.
-narrateur|Une autre goutte tombe.
-narrateur|La terre sent fort.
-papa|Tu veux encore verser, Mila ?
+narrateur|Aniss tient l'anse, plus près.
+narrateur|Mila verse un peu, cette fois.
+enfant-f|Ploc.
+copain|Ploc.
+papa|Tu vois, la sauge ?
+enfant-f|Oui, papa.
+maman|Elle boit, Aniss ?
+copain|Un peu.
+narrateur|Mila verse, sans se presser.
+narrateur|Aniss suit le seau des yeux.
+narrateur|La terre devient plus sombre.
+copain|Un.
+enfant-f|Deux.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de la sauge ?
 enfant-f|Oui.
-narrateur|Mila verse.
-narrateur|Aniss attend.
-maman|Chacun son tour.
-narrateur|Un oiseau chante tout près.
-papa|Tu l'as entendu ?
-enfant-f|Oui, papa.
-narrateur|Le ver de terre n'est plus là.
-narrateur|La terre a un petit trou brillant.
-enfant-f|Il est rentré.
-papa|Il a de l'eau, maintenant.</t>
+maman|Tes mains sont mouillées, Mila ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1789,17 +1823,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range le seau ? Oui. Maman tend la main. Mila et Aniss rangent le seau. Vous avez les mains froides ? Un peu. On essuie. La sauge brille encore. Elle a bu. Avec le seau rouge. Le seau sèche à l'envers. Une goutte tombe du bord. Ploc. Une dernière, pour la terre.</t>
+          <t>Aniss lève le seau trop haut. L'eau penche vers le bord. Tout d'un coup ! Il veut verser tout, tout de suite. Ça va trop ! Une vague part vers la terre. La sauge se couche un peu. Elle se couche ! Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le linge qui goutte. Sur la feuille, un éclat de sauge luit. Là, sur la sauge. Tu verses un peu, Aniss ? Aniss ne dit rien. Il souffle, puis baisse le seau. Oui. On verse juste un peu ? Oui, papa. Le seau sent la terre mouillée. L'eau tombe goutte à goutte. Mila pose le seau près d'Aniss. Aniss le rend, sans sauter. Ploc. Ploc. La sauge a bu, Mila ? Oui, papa. Le linge est lourd, Aniss ? Un peu. Ils se passent le seau, tout près. La terre chatouille les genoux. C'est plus facile. Le seau est moins lourd ? Oui, papa. Un rayon passe sur la sauge. Il allume la feuille.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range le seau ? Oui. Maman tend la main. Mila et Aniss rangent le seau. Vous avez les mains froides ? Un peu. On essuie. La sauge brille encore. Elle a bu. Avec le seau rouge. Le seau sèche à l'envers. Une goutte tombe du bord. Ploc. Une dernière, pour la terre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss lève le seau trop haut. L'eau penche vers le bord. Tout d'un coup ! Il veut verser tout, tout de suite. Ça va trop ! Une vague part vers la terre. La sauge se couche un peu. Elle se couche ! Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le linge qui goutte. Sur la feuille, un &lt;emphasis level="moderate"&gt;éclat de sauge&lt;/emphasis&gt; luit. Là, sur la sauge. Tu verses un peu, Aniss ? Aniss ne dit rien. Il souffle, puis baisse le seau. Oui. On verse juste un peu ? Oui, papa. Le seau sent la terre mouillée. L'eau tombe goutte à goutte. Mila pose le seau près d'Aniss. Aniss le rend, sans sauter. Ploc. Ploc. La sauge a bu, Mila ? Oui, papa. Le linge est lourd, Aniss ? Un peu. Ils se passent le seau, tout près. La terre chatouille les genoux. C'est plus facile. Le seau est moins lourd ? Oui, papa. Un rayon passe sur la sauge. Il allume la feuille.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maman tend la &lt;emphasis&gt;main&lt;/emphasis&gt;. Tania et Ulysse rangent le seau.&lt;/slow&gt; [pause]</t>
+          <t>Aniss lève le seau trop haut. L'eau penche vers le bord. Tout d'un coup ! Il veut verser tout, tout de suite. Ça va trop ! Une vague part vers la terre. La sauge se couche un peu. Elle se couche ! Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le linge qui goutte. Sur la feuille, un &lt;emphasis&gt;éclat de sauge&lt;/emphasis&gt; luit. Là, sur la sauge. Tu verses un peu, Aniss ? Aniss ne dit rien. Il souffle, puis baisse le seau. Oui. On verse juste un peu ? Oui, papa. Le seau sent la terre mouillée. L'eau tombe goutte à goutte. Mila pose le seau près d'Aniss. Aniss le rend, sans sauter. Ploc. Ploc. La sauge a bu, Mila ? Oui, papa. Le linge est lourd, Aniss ? Un peu. Ils se passent le seau, tout près. La terre chatouille les genoux. C'est plus facile. Le seau est moins lourd ? Oui, papa. Un rayon passe sur la sauge. Il allume la feuille. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,18 +1880,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1880,30 +1914,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de sauge</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1912,10 +1946,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1924,25 +1958,60 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_veut_verser_tout_elle_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On range le seau ?
-enfant-f|Oui.
-narrateur|Maman tend la main.
-narrateur|Mila et Aniss rangent le seau.
-papa|Vous avez les mains froides ?
-enfant-f|Un peu.
-papa|On essuie.
-narrateur|La sauge brille encore.
-maman|Elle a bu.
-enfant-f|Avec le seau rouge.
-narrateur|Le seau sèche à l'envers.
-narrateur|Une goutte tombe du bord.
-narrateur|Ploc.
-maman|Une dernière, pour la terre.</t>
+          <t>narrateur|Aniss lève le seau trop haut.
+narrateur|L'eau penche vers le bord.
+copain|Tout d'un coup !
+narrateur|Il veut verser tout, tout de suite.
+enfant-f|Ça va trop !
+narrateur|Une vague part vers la terre.
+narrateur|La sauge se couche un peu.
+enfant-f|Elle se couche !
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le seau, un instant.
+narrateur|Elle écoute le linge qui goutte.
+narrateur|Sur la feuille, un éclat de sauge luit.
+enfant-f|Là, sur la sauge.
+enfant-f|Tu verses un peu, Aniss ?
+narrateur|Aniss ne dit rien.
+narrateur|Il souffle, puis baisse le seau.
+copain|Oui.
+papa|On verse juste un peu ?
+enfant-f|Oui, papa.
+narrateur|Le seau sent la terre mouillée.
+narrateur|L'eau tombe goutte à goutte.
+narrateur|Mila pose le seau près d'Aniss.
+narrateur|Aniss le rend, sans sauter.
+enfant-f|Ploc.
+copain|Ploc.
+papa|La sauge a bu, Mila ?
+enfant-f|Oui, papa.
+maman|Le linge est lourd, Aniss ?
+copain|Un peu.
+narrateur|Ils se passent le seau, tout près.
+narrateur|La terre chatouille les genoux.
+enfant-f|C'est plus facile.
+papa|Le seau est moins lourd ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur la sauge.
+enfant-f|Il allume la feuille.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1969,17 +2038,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La sauge est brillante. Le seau rouge sèche. La terre est contente. Moi aussi.</t>
+          <t>Ils restent près de la sauge. Maman essuie un peu d'eau. La sauge a bu, papa. Tu l'as vue, toi ? Oui, près du bac. On est bien, ici. Mila tapote le seau du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le seau est resté, Mila. Oui, avec Aniss. Le seau est resté. Ça sent la sauge, un peu froide. Et le linge, maman. Oui, dans l'air. Le seau sèche à l'envers. Un éclat de sauge tient sur la feuille.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La sauge est brillante. Le seau rouge sèche. La terre est contente. Moi aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la sauge. Maman essuie un peu d'eau. La sauge a bu, papa. Tu l'as vue, toi ? Oui, près du bac. On est bien, ici. Mila tapote le seau du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le seau est resté, Mila. Oui, avec Aniss. Le seau est resté. Ça sent la sauge, un peu froide. Et le linge, maman. Oui, dans l'air. Le seau sèche à l'envers. Un &lt;emphasis level="moderate"&gt;éclat de sauge&lt;/emphasis&gt; tient sur la feuille.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la sauge. Maman essuie un peu d'eau. La sauge a bu, papa. Tu l'as vue, toi ? Oui, près du bac. On est bien, ici. Mila tapote le seau du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le seau est resté, Mila. Oui, avec Aniss. Le seau est resté. Ça sent la sauge, un peu froide. Et le linge, maman. Oui, dans l'air. Le seau sèche à l'envers. Un &lt;emphasis&gt;éclat de sauge&lt;/emphasis&gt; tient sur la feuille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2026,7 +2095,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2034,10 +2103,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2046,12 +2115,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2060,14 +2129,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de sauge</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2079,11 +2152,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2092,27 +2165,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_feuille; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La sauge est brillante.
-narrateur|Le seau rouge sèche.
-papa|La terre est contente.
-enfant-f|Moi aussi.</t>
+          <t>narrateur|Ils restent près de la sauge.
+narrateur|Maman essuie un peu d'eau.
+enfant-f|La sauge a bu, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, près du bac.
+maman|On est bien, ici.
+narrateur|Mila tapote le seau du doigt.
+enfant-f|Il a une trace d'eau.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le seau est resté, Mila.
+enfant-f|Oui, avec Aniss.
+copain|Le seau est resté.
+narrateur|Ça sent la sauge, un peu froide.
+enfant-f|Et le linge, maman.
+maman|Oui, dans l'air.
+narrateur|Le seau sèche à l'envers.
+narrateur|Un éclat de sauge tient sur la feuille.</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2309,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>